<commit_message>
Refactor: monolithic → modular structure + add new data
</commit_message>
<xml_diff>
--- a/data_clean/output_wp.xlsx
+++ b/data_clean/output_wp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Documents\All Work Files\1. PE New Report\data_clean\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C54B68-15F7-4194-8078-AD98A2AA7CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35415E21-D936-4D79-B511-3769A0BF9A3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23507,7 +23507,7 @@
         <v>22</v>
       </c>
       <c r="L306" t="s">
-        <v>929</v>
+        <v>322</v>
       </c>
       <c r="M306" t="s">
         <v>22</v>
@@ -37395,7 +37395,7 @@
         <v>22</v>
       </c>
       <c r="L554" t="s">
-        <v>1632</v>
+        <v>90</v>
       </c>
       <c r="M554" t="s">
         <v>22</v>

</xml_diff>